<commit_message>
implementing AI decision making
</commit_message>
<xml_diff>
--- a/src/beastmistress/assets/data/beasts.xlsx
+++ b/src/beastmistress/assets/data/beasts.xlsx
@@ -15,32 +15,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="60">
   <si>
     <t>Species Name</t>
   </si>
   <si>
-    <t>Physical Attack</t>
-  </si>
-  <si>
-    <t>Physical Defence</t>
-  </si>
-  <si>
-    <t>Magical Attack</t>
-  </si>
-  <si>
-    <t>Magical Defence</t>
-  </si>
-  <si>
     <t>Vitality</t>
   </si>
   <si>
-    <t>Speed</t>
-  </si>
-  <si>
-    <t>Luck</t>
-  </si>
-  <si>
     <t>Total</t>
   </si>
   <si>
@@ -101,9 +83,6 @@
     <t>Feth</t>
   </si>
   <si>
-    <t>Regen Rate</t>
-  </si>
-  <si>
     <t>Piety</t>
   </si>
   <si>
@@ -189,6 +168,33 @@
   </si>
   <si>
     <t>Dark/Light</t>
+  </si>
+  <si>
+    <t>Celerity</t>
+  </si>
+  <si>
+    <t>Fortune</t>
+  </si>
+  <si>
+    <t>Aggressiveness</t>
+  </si>
+  <si>
+    <t>Willpower</t>
+  </si>
+  <si>
+    <t>Toughness</t>
+  </si>
+  <si>
+    <t>Determination</t>
+  </si>
+  <si>
+    <t>Conviction</t>
+  </si>
+  <si>
+    <t>Debug</t>
+  </si>
+  <si>
+    <t>DebugBeast</t>
   </si>
 </sst>
 </file>
@@ -597,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -616,120 +622,120 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="B2" s="1">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D2" s="1">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E2" s="1">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F2" s="1">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G2" s="1">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="H2" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I2" s="1">
-        <v>10</v>
+        <v>9999</v>
       </c>
       <c r="J2" s="1">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="K2" s="1">
         <f>SUM(B2:J2)</f>
-        <v>120</v>
+        <v>10007</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B3" s="1">
         <v>10</v>
       </c>
       <c r="C3" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1">
         <v>20</v>
       </c>
       <c r="E3" s="1">
+        <v>20</v>
+      </c>
+      <c r="F3" s="1">
+        <v>10</v>
+      </c>
+      <c r="G3" s="1">
         <v>15</v>
-      </c>
-      <c r="F3" s="1">
-        <v>15</v>
-      </c>
-      <c r="G3" s="1">
-        <v>10</v>
       </c>
       <c r="H3" s="1">
         <v>5</v>
       </c>
       <c r="I3" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J3" s="1">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K3" s="1">
-        <f t="shared" ref="K3:K4" si="0">SUM(B3:J3)</f>
+        <f>SUM(B3:J3)</f>
         <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B4" s="1">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C4" s="1">
         <v>15</v>
       </c>
       <c r="D4" s="1">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E4" s="1">
         <v>15</v>
@@ -744,12 +750,48 @@
         <v>5</v>
       </c>
       <c r="I4" s="1">
+        <v>15</v>
+      </c>
+      <c r="J4" s="1">
+        <v>15</v>
+      </c>
+      <c r="K4" s="1">
+        <f t="shared" ref="K4:K5" si="0">SUM(B4:J4)</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1">
+        <v>20</v>
+      </c>
+      <c r="C5" s="1">
+        <v>15</v>
+      </c>
+      <c r="D5" s="1">
         <v>10</v>
       </c>
-      <c r="J4" s="1">
+      <c r="E5" s="1">
+        <v>15</v>
+      </c>
+      <c r="F5" s="1">
+        <v>15</v>
+      </c>
+      <c r="G5" s="1">
+        <v>10</v>
+      </c>
+      <c r="H5" s="1">
+        <v>5</v>
+      </c>
+      <c r="I5" s="1">
+        <v>10</v>
+      </c>
+      <c r="J5" s="1">
         <v>20</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K5" s="1">
         <f t="shared" si="0"/>
         <v>120</v>
       </c>
@@ -761,7 +803,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AK2"/>
+  <dimension ref="A1:AK3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="9" width="8.88671875" style="1"/>
@@ -774,141 +816,149 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="I1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="J1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>